<commit_message>
Revise the program listings spreadsheet
Renames the link issue column to GS Website Titles, drops the
destination checked column, and puts the read me tab first.

The read me now carries the findings that have no row in the
chart: the catalog cycle, the five programs with no settled Fall
2027 status, the unpublished directory page, the International
Programs document, the prospective students page groupings, the
contact block, and the unopened tile destinations.
</commit_message>
<xml_diff>
--- a/committee/grad-facilitator/documents/graduate-program-listings.xlsx
+++ b/committee/grad-facilitator/documents/graduate-program-listings.xlsx
@@ -7,11 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="programs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="read me" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="read me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="programs" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'programs'!$A$1:$J$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'programs'!$A$1:$I$54</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,7 +32,7 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="006E1F2A"/>
-      <sz val="10"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -41,15 +41,27 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
       <color rgb="006E1F2A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001B1C1E"/>
       <sz val="10"/>
-      <u val="single"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="006E1F2A"/>
-      <sz val="11"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="006E1F2A"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="4">
@@ -92,9 +104,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -103,7 +133,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -112,14 +142,8 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -486,7 +510,253 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:B22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>graduate program listings</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Every graduate program in the 2026-2027 catalog and every tile on the Office of Graduate Studies page, in one list. See the programs tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Compiled 10 September 2026 by I. Thiebaut.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n"/>
+      <c r="B4" s="2" t="n"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>columns</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>in catalog</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Whether the program appears in the 2026-2027 catalog. The three rows that do not are tinted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>on tiles</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Whether the program has a tile. "unresolved" marks Mathematics, Single Subject Matter Preparation, where the tiles carry Mathematics, Single Subject Matter and Foundational Mathematics, Single Subject and which names which is an open question.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>GS Website Titles</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>What the Graduate Studies tile does that needs a look: a shared link, a different name, an archived catalog year. Blank means nothing noted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>What the catalog says about the program, including concentrations and tracks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n"/>
+      <c r="B10" s="2" t="n"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>findings not in the chart</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>catalog cycle</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>The 2026-2027 catalog is current and there is no 2027-2028 catalog. Fall 2027 status for any program comes from the department rather than from the catalog.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>English, M.A.</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>In neither the catalog nor the tiles. The International Programs document records it as suspended until Fall 2026. The department’s graduate page is live under the heading “New M.A. in English at CSU East Bay” and advertises applications for Fall 2024 through Cal State Apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Art, M.A.</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>In neither the catalog nor the tiles, and linked from the prospective graduate students page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Communication, M.A.</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>In the catalog, absent from the tiles, recorded as suspended. Held out of the programs tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>M.B.A., Global Innovators</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Recorded in the International Programs document as not accepting applications for Fall 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>eLearning certificates</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>eLearning Administration, eLearning Design, and eLearning Technology appear on the unpublished graduate program directory page and on no other page found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>unpublished directory page</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>/graduate-studies/graduate-program-directory.html is tagged “Unused page. Do not publish.” and is live. The prospective graduate students page sends applicants there for program coordinator contacts. It carries no Music tile and links into catalog years 33 and 39.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>International Programs document</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>The admission requirements PDF is stamped “Information verified 7/15/2025”. It carries the English M.A. as suspended until Fall 2026, the Global Innovators M.B.A. as not accepting for Fall 2026, and the Computer Science GRE as waived for Fall 2025 and Spring 2026. International applicants for Fall 2027 read this document.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>prospective students page</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>The department list runs under a College of Education and Allied Studies heading. Kinesiology, Nursing, Speech Language and Hearing Sciences, and Social Work are College of Health. Hospitality, Recreation and Tourism is CLASS. Special Education has no entry. Biological Sciences links to a Blogspot site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>contact block</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Divya Sitaraman’s email is listed as joshua.kerr@csueastbay.edu. The graduate recruitment facilitator is listed as a Graduate Student Success Facilitator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>tile destinations</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>The tile links have not been opened, except Accountancy, which reaches the MS in Accountancy program page.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -498,2347 +768,2284 @@
     <col width="46" customWidth="1" min="7" max="7"/>
     <col width="44" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>college</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>department</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>program</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>in catalog</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>on tiles</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>catalog link</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>tile link</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>link issue</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t>GS Website Titles</t>
+        </is>
+      </c>
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>destination checked</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>Graduate School of Education</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>Post-baccalaureate Health Professions Academic Program Certificate</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F2" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20603&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/phaprogram/</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>tile is named Pre-Professional Health Academic Program (PHAP)</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="8" t="inlineStr">
         <is>
           <t>self-support only, delivered through university extension, placed here provisionally, department to confirm</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Educational Leadership</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>Educational Leadership, M.S.</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20452&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/el/programs/master-in-el.html</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="H3" s="8" t="inlineStr"/>
+      <c r="I3" s="8" t="inlineStr">
         <is>
           <t>tracks: with PASC, with optional PASC</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>Educational Leadership</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>Educational Leadership, Ed.D.</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20451&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/edd/index.html</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="H4" s="8" t="inlineStr"/>
+      <c r="I4" s="8" t="inlineStr">
         <is>
           <t>summer admission</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Educational Leadership</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Preliminary Administrative Services Credential</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20497&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/el/programs/prelim-admin-services.html</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="H5" s="8" t="inlineStr"/>
+      <c r="I5" s="8" t="inlineStr">
         <is>
           <t>available self-support</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Educational Leadership</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>Administrative Services Credential, Clear Induction</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr"/>
+      <c r="G6" s="13" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/el/programs/clear-admin-services-cred.html</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="11" t="inlineStr">
         <is>
           <t>tile only</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I6" s="11" t="inlineStr">
         <is>
           <t>not in the catalog</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Educational Psychology</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Counseling Psychology, M.S.</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20476&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/epsy/graduate-programs/index.html</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" s="8" t="inlineStr">
         <is>
           <t>one tile, named Counseling, for all three concentrations</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I7" s="8" t="inlineStr">
         <is>
           <t>concentrations: Marriage and Family Therapy, School Counseling, School Psychology</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Educational Psychology</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>PPS Credential, School Counseling</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20509&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/epsy/graduate-programs/school-counseling.html</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
+      <c r="H8" s="8" t="inlineStr"/>
+      <c r="I8" s="8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Educational Psychology</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>PPS Credential, School Psychology</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20508&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/school-psychology/prospective-students.html</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
+      <c r="H9" s="8" t="inlineStr"/>
+      <c r="I9" s="8" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Teacher Education</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Curriculum and Instruction, M.S.</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20641&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G10" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/ted/programs-admissions/masters/index.html</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" s="8" t="inlineStr">
         <is>
           <t>shared with Early Childhood Education and Educational Technology</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
+      <c r="I10" s="8" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Teacher Education</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Early Childhood Education, M.S.</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20502&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G11" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/ted/programs-admissions/masters/index.html</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" s="8" t="inlineStr">
         <is>
           <t>shared with Curriculum and Instruction and Educational Technology</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr"/>
+      <c r="I11" s="8" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Teacher Education</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>Educational Technology, M.S.</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20565&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G12" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/ted/programs-admissions/masters/index.html</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H12" s="8" t="inlineStr">
         <is>
           <t>shared with Curriculum and Instruction and Early Childhood Education</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr"/>
+      <c r="I12" s="8" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Teacher Education</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Reading and Literacy, M.S.</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20600&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G13" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/ted/programs-admissions/masters/reading-cert1.html</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="H13" s="8" t="inlineStr"/>
+      <c r="I13" s="8" t="inlineStr">
         <is>
           <t>self-support only</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Teacher Education</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>Multiple Subject Credential</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20499&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G14" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/cssc/prospective-cred-student/multiple-subject.html</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H14" s="8" t="inlineStr">
         <is>
           <t>tile is named Multi-subject Teaching</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr"/>
+      <c r="I14" s="8" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Teacher Education</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Single Subject Credential</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20503&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G15" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/cssc/prospective-cred-student/single-subject.html</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H15" s="8" t="inlineStr">
         <is>
           <t>tile is named Single-subject Teaching</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="inlineStr"/>
+      <c r="I15" s="8" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>Teacher Education</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>Educational Technology Certificate</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20610&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="G16" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=39&amp;poid=18263&amp;returnto=36991</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H16" s="8" t="inlineStr">
         <is>
           <t>points into catalog year 39; the current catalog is 44</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr"/>
+      <c r="I16" s="8" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Special Education</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>Special Education, M.S.</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20561&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G17" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/cssc/prospective-cred-student/special-education.html</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H17" s="8" t="inlineStr">
         <is>
           <t>shared with the Education Specialist Credential</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I17" s="8" t="inlineStr">
         <is>
           <t>concentrations: Extensive Support Needs, Mild/Moderate Support Needs</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Special Education</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>Education Specialist Credential</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20601&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="G18" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/cssc/prospective-cred-student/special-education.html</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H18" s="8" t="inlineStr">
         <is>
           <t>shared with Special Education, M.S.</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="inlineStr"/>
+      <c r="I18" s="8" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Art</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>Interaction Design and Interactive Art, M.A.</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20423&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G19" s="10" t="inlineStr">
         <is>
           <t>https://ixdia.org</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H19" s="8" t="inlineStr">
         <is>
           <t>off site; tile is named Interaction Design</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr"/>
-      <c r="J19" s="2" t="inlineStr"/>
+      <c r="I19" s="8" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>Art</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>Interaction and User Experience Design Certificate</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F20" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20693&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="G20" s="9" t="inlineStr"/>
+      <c r="H20" s="8" t="inlineStr">
         <is>
           <t>no tile</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr"/>
+      <c r="I20" s="8" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>History, M.A.</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20697&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="G21" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/history/degree-programs/ma-degree-programs_new.html</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr"/>
-      <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" s="2" t="inlineStr"/>
+      <c r="H21" s="8" t="inlineStr"/>
+      <c r="I21" s="8" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>Social Science Single Subject Matter Preparation</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="F22" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20612&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="G22" s="9" t="inlineStr"/>
+      <c r="H22" s="8" t="inlineStr">
         <is>
           <t>no tile</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr"/>
+      <c r="I22" s="8" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>Hospitality, Recreation and Tourism</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Hospitality, Recreation and Tourism, M.S.</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20485&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G23" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/hrt/grad/index.html</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr"/>
-      <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="2" t="inlineStr"/>
+      <c r="H23" s="8" t="inlineStr"/>
+      <c r="I23" s="8" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>Music</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
         <is>
           <t>Music, M.A.</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20498&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="G24" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/music/prospective/ma.html</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="2" t="inlineStr"/>
+      <c r="H24" s="8" t="inlineStr"/>
+      <c r="I24" s="8" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>Music</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>Music Single Subject Matter Preparation Certificate</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20615&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
+      <c r="G25" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/music/prospective/music-ed.html</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr"/>
-      <c r="I25" s="2" t="inlineStr"/>
-      <c r="J25" s="2" t="inlineStr"/>
+      <c r="H25" s="8" t="inlineStr"/>
+      <c r="I25" s="8" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>Public Affairs and Administration</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>Health Care Administration, M.S.</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20664&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr">
+      <c r="G26" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/paa/healthcare/index.html</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" s="2" t="inlineStr"/>
+      <c r="H26" s="8" t="inlineStr"/>
+      <c r="I26" s="8" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>College of Letters, Arts, and Social Sciences</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>Public Affairs and Administration</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>Public Administration, M.P.A.</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20490&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G27" s="4" t="inlineStr">
+      <c r="G27" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/paa/public-admin/index.html</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr"/>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="H27" s="8" t="inlineStr"/>
+      <c r="I27" s="8" t="inlineStr">
         <is>
           <t>concentrations: Health Care Administration, Public Management and Policy Analysis</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>College of Science</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>Biological Sciences</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
         <is>
           <t>Biological Science, M.S.</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20488&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
+      <c r="G28" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/biology/graduate-program/biology-ms-program/index.html</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="2" t="inlineStr"/>
+      <c r="H28" s="8" t="inlineStr"/>
+      <c r="I28" s="8" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>College of Science</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>Biological Sciences</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr">
         <is>
           <t>Marine Science, M.S.</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20542&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G29" s="4" t="inlineStr">
+      <c r="G29" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/biology/graduate-program/ms-in-marine-sciences.html</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr"/>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="H29" s="8" t="inlineStr"/>
+      <c r="I29" s="8" t="inlineStr">
         <is>
           <t>administered by Moss Landing Marine Laboratories</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>College of Science</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>Biological Sciences</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>Biotechnology Certificate</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20599&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G30" s="4" t="inlineStr">
+      <c r="G30" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/biology/graduate-program/biotechnology-certificate-program-bcp/index.html</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
-      <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="2" t="inlineStr"/>
+      <c r="H30" s="8" t="inlineStr"/>
+      <c r="I30" s="8" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>College of Science</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>Chemistry and Biochemistry</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>Chemistry, M.S.</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20540&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G31" s="4" t="inlineStr">
+      <c r="G31" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/chemistry/graduate/index.html</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr"/>
-      <c r="I31" s="2" t="inlineStr">
+      <c r="H31" s="8" t="inlineStr"/>
+      <c r="I31" s="8" t="inlineStr">
         <is>
           <t>concentrations: Chemistry, Biochemistry</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>College of Science</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>Computer Science</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C32" s="8" t="inlineStr">
         <is>
           <t>Computer Science, M.S.</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20563&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G32" s="4" t="inlineStr">
+      <c r="G32" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/cs/degrees-programs1/index.html</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="H32" s="8" t="inlineStr"/>
+      <c r="I32" s="8" t="inlineStr">
         <is>
           <t>concentrations: Artificial Intelligence and Machine Learning, Computer Networks, Computer Science</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>College of Science</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>Earth and Environmental Sciences</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
         <is>
           <t>Environmental Geosciences, M.S.</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20479&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G33" s="4" t="inlineStr">
+      <c r="G33" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/earth/graduate-program/index.html</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr"/>
-      <c r="I33" s="2" t="inlineStr"/>
-      <c r="J33" s="2" t="inlineStr"/>
+      <c r="H33" s="8" t="inlineStr"/>
+      <c r="I33" s="8" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>College of Science</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>Engineering</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C34" s="8" t="inlineStr">
         <is>
           <t>Construction Management, M.S.</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20474&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr">
+      <c r="G34" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/engineering/programs-degrees/graduate-degrees.html</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="H34" s="8" t="inlineStr">
         <is>
           <t>shared with Engineering Management</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr"/>
-      <c r="J34" s="2" t="inlineStr"/>
+      <c r="I34" s="8" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>College of Science</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>Engineering</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C35" s="8" t="inlineStr">
         <is>
           <t>Engineering Management, M.S.</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20475&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G35" s="4" t="inlineStr">
+      <c r="G35" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/engineering/programs-degrees/graduate-degrees.html</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="H35" s="8" t="inlineStr">
         <is>
           <t>shared with Construction Management</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr"/>
-      <c r="J35" s="2" t="inlineStr"/>
+      <c r="I35" s="8" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>College of Science</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B36" s="8" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C36" s="8" t="inlineStr">
         <is>
           <t>Mathematics, M.S.</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F36" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20496&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G36" s="4" t="inlineStr">
+      <c r="G36" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/math/degrees-and-programs/index.html</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="H36" s="8" t="inlineStr">
         <is>
           <t>shared with the Foundational Mathematics and Mathematics Single Subject Matter tiles</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr"/>
-      <c r="J36" s="2" t="inlineStr"/>
+      <c r="I36" s="8" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>College of Science</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B37" s="8" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C37" s="8" t="inlineStr">
         <is>
           <t>Mathematics, Single Subject Matter Certificate</t>
         </is>
       </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F37" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20624&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G37" s="4" t="inlineStr">
+      <c r="G37" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/math/degrees-and-programs/index.html</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H37" s="8" t="inlineStr">
         <is>
           <t>tile is named Mathematics, Single Subject Matter; shared with Mathematics, M.S. and the Foundational Mathematics tile</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr"/>
-      <c r="J37" s="2" t="inlineStr"/>
+      <c r="I37" s="8" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>College of Science</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B38" s="8" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C38" s="8" t="inlineStr">
         <is>
           <t>Mathematics, Single Subject Matter Preparation</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="inlineStr">
         <is>
           <t>unresolved</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="F38" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20623&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G38" s="3" t="inlineStr"/>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="G38" s="9" t="inlineStr"/>
+      <c r="H38" s="8" t="inlineStr">
         <is>
           <t>the tiles carry Mathematics, Single Subject Matter and Foundational Mathematics, Single Subject; which of the two catalog entries each names is an open question</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr"/>
-      <c r="J38" s="2" t="inlineStr"/>
+      <c r="I38" s="8" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="A39" s="11" t="inlineStr">
         <is>
           <t>College of Science</t>
         </is>
       </c>
-      <c r="B39" s="5" t="inlineStr">
+      <c r="B39" s="11" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="C39" s="5" t="inlineStr">
+      <c r="C39" s="11" t="inlineStr">
         <is>
           <t>Foundational Mathematics, Single Subject</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="D39" s="12" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="inlineStr"/>
-      <c r="G39" s="7" t="inlineStr">
+      <c r="E39" s="12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F39" s="12" t="inlineStr"/>
+      <c r="G39" s="13" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/math/degrees-and-programs/index.html</t>
         </is>
       </c>
-      <c r="H39" s="5" t="inlineStr">
+      <c r="H39" s="11" t="inlineStr">
         <is>
           <t>tile only; shared with Mathematics, M.S. and the Mathematics Single Subject Matter tile</t>
         </is>
       </c>
-      <c r="I39" s="5" t="inlineStr">
+      <c r="I39" s="11" t="inlineStr">
         <is>
           <t>not in the catalog under this name; the Mathematics degrees and programs page lists no foundational-level program</t>
         </is>
       </c>
-      <c r="J39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>College of Science</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B40" s="8" t="inlineStr">
         <is>
           <t>Statistics and Biostatistics</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C40" s="8" t="inlineStr">
         <is>
           <t>Statistics, M.S.</t>
         </is>
       </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F40" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20604&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G40" s="4" t="inlineStr">
+      <c r="G40" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/statistics/degrees-programs/index.html</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="H40" s="8" t="inlineStr">
         <is>
           <t>shared with the Applied Statistics and Theoretical Statistics tiles</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr">
+      <c r="I40" s="8" t="inlineStr">
         <is>
           <t>concentrations: Actuarial Science, Applied Statistics, Biostatistics, Data Science, Mathematical Statistics</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>College of Science</t>
         </is>
       </c>
-      <c r="B41" s="2" t="inlineStr">
+      <c r="B41" s="8" t="inlineStr">
         <is>
           <t>Statistics and Biostatistics</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
+      <c r="C41" s="8" t="inlineStr">
         <is>
           <t>Applied Statistics Certificate</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F41" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20621&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G41" s="4" t="inlineStr">
+      <c r="G41" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/statistics/degrees-programs/index.html</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="H41" s="8" t="inlineStr">
         <is>
           <t>shared with Statistics, M.S. and the Theoretical Statistics tile</t>
         </is>
       </c>
-      <c r="I41" s="2" t="inlineStr"/>
-      <c r="J41" s="2" t="inlineStr"/>
+      <c r="I41" s="8" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>College of Science</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B42" s="8" t="inlineStr">
         <is>
           <t>Statistics and Biostatistics</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C42" s="8" t="inlineStr">
         <is>
           <t>Theoretical Statistics Certificate</t>
         </is>
       </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F42" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20622&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G42" s="4" t="inlineStr">
+      <c r="G42" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/statistics/degrees-programs/index.html</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="H42" s="8" t="inlineStr">
         <is>
           <t>shared with Statistics, M.S. and the Applied Statistics tile</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr"/>
-      <c r="J42" s="2" t="inlineStr"/>
+      <c r="I42" s="8" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="A43" s="11" t="inlineStr">
         <is>
           <t>College of Science</t>
         </is>
       </c>
-      <c r="B43" s="5" t="inlineStr">
+      <c r="B43" s="11" t="inlineStr">
         <is>
           <t>Statistics and Biostatistics</t>
         </is>
       </c>
-      <c r="C43" s="5" t="inlineStr">
+      <c r="C43" s="11" t="inlineStr">
         <is>
           <t>Biostatistics</t>
         </is>
       </c>
-      <c r="D43" s="6" t="inlineStr">
+      <c r="D43" s="12" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="E43" s="6" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="inlineStr"/>
-      <c r="G43" s="7" t="inlineStr">
+      <c r="E43" s="12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F43" s="12" t="inlineStr"/>
+      <c r="G43" s="13" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/statistics/biostatistics-psm/index.html</t>
         </is>
       </c>
-      <c r="H43" s="5" t="inlineStr">
+      <c r="H43" s="11" t="inlineStr">
         <is>
           <t>tile only</t>
         </is>
       </c>
-      <c r="I43" s="5" t="inlineStr">
+      <c r="I43" s="11" t="inlineStr">
         <is>
           <t>not in the catalog as a separate program; carried as a Statistics concentration</t>
         </is>
       </c>
-      <c r="J43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>College of Business and Economics</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B44" s="8" t="inlineStr">
         <is>
           <t>Accounting and Finance</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C44" s="8" t="inlineStr">
         <is>
           <t>Accountancy, M.S.</t>
         </is>
       </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F44" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20440&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G44" s="4" t="inlineStr">
+      <c r="G44" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/msa/index.html</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="H44" s="8" t="inlineStr">
         <is>
           <t>opened; reaches the MS in Accountancy program page</t>
         </is>
       </c>
-      <c r="I44" s="2" t="inlineStr">
+      <c r="I44" s="8" t="inlineStr">
         <is>
           <t>self-support only</t>
         </is>
       </c>
-      <c r="J44" s="2" t="inlineStr">
-        <is>
-          <t>yes, reaches the MS in Accountancy program page</t>
-        </is>
-      </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>College of Business and Economics</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B45" s="8" t="inlineStr">
         <is>
           <t>Economics</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C45" s="8" t="inlineStr">
         <is>
           <t>Quantitative Economics, M.S.</t>
         </is>
       </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="inlineStr">
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="F45" s="4" t="inlineStr">
+      <c r="F45" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20653&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G45" s="3" t="inlineStr"/>
-      <c r="H45" s="2" t="inlineStr">
+      <c r="G45" s="9" t="inlineStr"/>
+      <c r="H45" s="8" t="inlineStr">
         <is>
           <t>no tile</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr"/>
-      <c r="J45" s="2" t="inlineStr"/>
+      <c r="I45" s="8" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>College of Business and Economics</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B46" s="8" t="inlineStr">
         <is>
           <t>Management</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C46" s="8" t="inlineStr">
         <is>
           <t>Business Analytics, M.S.</t>
         </is>
       </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
+      <c r="D46" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F46" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20441&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G46" s="4" t="inlineStr">
+      <c r="G46" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/msba/index.html</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr"/>
-      <c r="I46" s="2" t="inlineStr"/>
-      <c r="J46" s="2" t="inlineStr"/>
+      <c r="H46" s="8" t="inlineStr"/>
+      <c r="I46" s="8" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>College of Business and Economics</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B47" s="8" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C47" s="8" t="inlineStr">
         <is>
           <t>Marketing Analytics, M.S.</t>
         </is>
       </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F47" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20675&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G47" s="4" t="inlineStr">
+      <c r="G47" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/msma/index.html</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr"/>
-      <c r="I47" s="2" t="inlineStr"/>
-      <c r="J47" s="2" t="inlineStr"/>
+      <c r="H47" s="8" t="inlineStr"/>
+      <c r="I47" s="8" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>College of Business and Economics</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B48" s="8" t="inlineStr">
         <is>
           <t>college-wide</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="C48" s="8" t="inlineStr">
         <is>
           <t>Business Administration, M.B.A.</t>
         </is>
       </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E48" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
+      <c r="D48" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F48" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20559&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G48" s="4" t="inlineStr">
+      <c r="G48" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/mba/index.html</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr"/>
-      <c r="I48" s="2" t="inlineStr">
+      <c r="H48" s="8" t="inlineStr"/>
+      <c r="I48" s="8" t="inlineStr">
         <is>
           <t>concentrations delivered across departments: Finance, General Business, General Business One-Year Accelerated (self-support), Human Resources Management and Organizational Behavior, Marketing Management, Operations and Supply Chain Management</t>
         </is>
       </c>
-      <c r="J48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>College of Health</t>
         </is>
       </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="B49" s="8" t="inlineStr">
         <is>
           <t>Kinesiology</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="C49" s="8" t="inlineStr">
         <is>
           <t>Kinesiology, M.S.</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F49" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20504&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G49" s="4" t="inlineStr">
+      <c r="G49" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/kin/programs/ms-kinesiology.html</t>
         </is>
       </c>
-      <c r="H49" s="2" t="inlineStr"/>
-      <c r="I49" s="2" t="inlineStr">
+      <c r="H49" s="8" t="inlineStr"/>
+      <c r="I49" s="8" t="inlineStr">
         <is>
           <t>concentrations: Human Movement and Sport Science, Physical Activity and Exercise</t>
         </is>
       </c>
-      <c r="J49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>College of Health</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B50" s="8" t="inlineStr">
         <is>
           <t>Kinesiology</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="C50" s="8" t="inlineStr">
         <is>
           <t>Physical Education Single Subject Matter Preparation</t>
         </is>
       </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E50" s="3" t="inlineStr">
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E50" s="9" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="F50" s="4" t="inlineStr">
+      <c r="F50" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20597&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G50" s="3" t="inlineStr"/>
-      <c r="H50" s="2" t="inlineStr">
+      <c r="G50" s="9" t="inlineStr"/>
+      <c r="H50" s="8" t="inlineStr">
         <is>
           <t>no tile</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr"/>
-      <c r="J50" s="2" t="inlineStr"/>
+      <c r="I50" s="8" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>College of Health</t>
         </is>
       </c>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="B51" s="8" t="inlineStr">
         <is>
           <t>Nursing</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
+      <c r="C51" s="8" t="inlineStr">
         <is>
           <t>Nursing, M.S.</t>
         </is>
       </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F51" s="4" t="inlineStr">
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E51" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F51" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20687&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G51" s="4" t="inlineStr">
+      <c r="G51" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/nursing/msn-programs/index.html</t>
         </is>
       </c>
-      <c r="H51" s="2" t="inlineStr"/>
-      <c r="I51" s="2" t="inlineStr"/>
-      <c r="J51" s="2" t="inlineStr"/>
+      <c r="H51" s="8" t="inlineStr"/>
+      <c r="I51" s="8" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>College of Health</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B52" s="8" t="inlineStr">
         <is>
           <t>Social Work</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
+      <c r="C52" s="8" t="inlineStr">
         <is>
           <t>Social Work, M.S.W.</t>
         </is>
       </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F52" s="4" t="inlineStr">
+      <c r="D52" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F52" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20686&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G52" s="4" t="inlineStr">
+      <c r="G52" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/sw/apply-to-msw.html</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr"/>
-      <c r="I52" s="2" t="inlineStr">
+      <c r="H52" s="8" t="inlineStr"/>
+      <c r="I52" s="8" t="inlineStr">
         <is>
           <t>tracks: standard, advanced standing</t>
         </is>
       </c>
-      <c r="J52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+      <c r="A53" s="8" t="inlineStr">
         <is>
           <t>College of Health</t>
         </is>
       </c>
-      <c r="B53" s="2" t="inlineStr">
+      <c r="B53" s="8" t="inlineStr">
         <is>
           <t>Speech, Language, and Hearing Sciences</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="C53" s="8" t="inlineStr">
         <is>
           <t>Speech-Language Pathology, M.S.</t>
         </is>
       </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E53" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F53" s="4" t="inlineStr">
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E53" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F53" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20533&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G53" s="4" t="inlineStr">
+      <c r="G53" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/slhs/masters-in-speech-language-pathology/index.html</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr">
+      <c r="H53" s="8" t="inlineStr">
         <is>
           <t>shared with the Speech Language Pathology Services credential tile</t>
         </is>
       </c>
-      <c r="I53" s="2" t="inlineStr"/>
-      <c r="J53" s="2" t="inlineStr"/>
+      <c r="I53" s="8" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>College of Health</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B54" s="8" t="inlineStr">
         <is>
           <t>Speech, Language, and Hearing Sciences</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="C54" s="8" t="inlineStr">
         <is>
           <t>Speech-Language Pathology Services Credential</t>
         </is>
       </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F54" s="4" t="inlineStr">
+      <c r="D54" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E54" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F54" s="10" t="inlineStr">
         <is>
           <t>https://catalog.csueastbay.edu/preview_program.php?catoid=44&amp;poid=20598&amp;returnto=42138</t>
         </is>
       </c>
-      <c r="G54" s="4" t="inlineStr">
+      <c r="G54" s="10" t="inlineStr">
         <is>
           <t>https://www.csueastbay.edu/slhs/masters-in-speech-language-pathology/index.html</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr">
+      <c r="H54" s="8" t="inlineStr">
         <is>
           <t>shared with Speech-Language Pathology, M.S.</t>
         </is>
       </c>
-      <c r="I54" s="2" t="inlineStr"/>
-      <c r="J54" s="2" t="inlineStr"/>
+      <c r="I54" s="8" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J54"/>
+  <autoFilter ref="A1:I54"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
@@ -2941,114 +3148,4 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="120" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="8" t="inlineStr">
-        <is>
-          <t>graduate program listings</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="9" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="9" t="inlineStr">
-        <is>
-          <t>Every graduate program in the 2026-2027 catalog and every tile on the Office of Graduate Studies page, in one list.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>Compiled 10 September 2026 by I. Thiebaut.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>columns</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>in catalog: whether the program appears in the 2026-2027 catalog. Rows tinted in the programs tab do not.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>on tiles: whether the program has a tile. "unresolved" marks Mathematics, Single Subject Matter Preparation, where the tiles carry Mathematics, Single Subject Matter and Foundational Mathematics, Single Subject and which names which is an open question.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>link issue: what the tile link does that needs a look. Blank means nothing noted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>note: what the catalog says about the program, including concentrations and tracks.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>destination checked: fill in as each tile link is opened. One is done.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>scope</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>The catalog and tile columns come from the catalog and the tile markup. Tile destinations are unopened except for Accountancy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>There is no 2027-2028 catalog yet, so Fall 2027 status for any program comes from the department, not from this list.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>